<commit_message>
frist try fix orchidia manuficture
</commit_message>
<xml_diff>
--- a/data/input/prevented_items/فاهس.xlsx
+++ b/data/input/prevented_items/فاهس.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\prevented_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F246886-BC9E-4906-9449-5E7D7D36D86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8303B5A1-51C4-4515-B7C5-7A355AFC97A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="305">
   <si>
     <t>كود</t>
   </si>
@@ -934,6 +934,12 @@
   </si>
   <si>
     <t>TADANERFI 20MG 4FILM</t>
+  </si>
+  <si>
+    <t>36804</t>
+  </si>
+  <si>
+    <t>CEREBROLYSIN AMP 1ML</t>
   </si>
 </sst>
 </file>
@@ -1271,7 +1277,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B313"/>
+  <dimension ref="A1:B314"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="31.85546875" customWidth="1"/>
@@ -3388,49 +3394,57 @@
         <v>115</v>
       </c>
     </row>
-    <row r="305" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B305" s="6" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="306" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B306" s="5" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="307" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B307" s="6" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="308" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B308" s="5" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="309" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B309" s="6" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="310" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B310" s="6" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="311" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B311" s="6" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="312" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B312" s="7" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="313" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B313" s="8" t="s">
         <v>302</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A314" t="s">
+        <v>303</v>
+      </c>
+      <c r="B314" t="s">
+        <v>304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add prevented item new
</commit_message>
<xml_diff>
--- a/data/input/prevented_items/فاهس.xlsx
+++ b/data/input/prevented_items/فاهس.xlsx
@@ -8,15 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\prevented_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC3E5BE-A80A-467A-9D51-162E492646DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D053A0-0FD4-424A-ADBD-8FEEF0E77357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-10410" windowWidth="16440" windowHeight="28320" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -25,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="457">
   <si>
     <t>كود</t>
   </si>
@@ -1354,13 +1365,55 @@
   </si>
   <si>
     <t>MENESTRO 1000 MG 20 CAPS</t>
+  </si>
+  <si>
+    <t>FEMAPENT 2.5MG 14 TABS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">هناك صنف اخر منه </t>
+  </si>
+  <si>
+    <t>MAALOX SUSP 250 ML</t>
+  </si>
+  <si>
+    <t>MAALOX PLUS FAST 180ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">صنفين بنفس السعر وله كودين موقوف لحين تصحيحه من المخزن </t>
+  </si>
+  <si>
+    <t xml:space="preserve">مش عوزينه </t>
+  </si>
+  <si>
+    <t xml:space="preserve">تاريخ </t>
+  </si>
+  <si>
+    <t>NEXIUM 40 MG 28 TABS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اكسبير </t>
+  </si>
+  <si>
+    <t>NANYMOM 30 TAB</t>
+  </si>
+  <si>
+    <t>LIDOCAINE 1 1 AMP 2 ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">تعليمات المدير </t>
+  </si>
+  <si>
+    <t>ROSUCHOLEST 20MG 20 TAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مفيش منه 20 قرص </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1390,6 +1443,12 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1466,7 +1525,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1485,6 +1544,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1681,11 +1744,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C494"/>
+  <dimension ref="A1:C502"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="65.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.5" x14ac:dyDescent="0.35">
@@ -6027,6 +6090,91 @@
         <v>437</v>
       </c>
     </row>
+    <row r="495" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A495">
+        <v>80691</v>
+      </c>
+      <c r="B495" t="s">
+        <v>443</v>
+      </c>
+      <c r="C495" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="496" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A496">
+        <v>86544</v>
+      </c>
+      <c r="B496" t="s">
+        <v>445</v>
+      </c>
+      <c r="C496" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="497" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A497">
+        <v>79694</v>
+      </c>
+      <c r="B497" t="s">
+        <v>446</v>
+      </c>
+      <c r="C497" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="498" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A498" s="10">
+        <v>47262</v>
+      </c>
+      <c r="B498" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="C498" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="499" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A499" s="10">
+        <v>78258</v>
+      </c>
+      <c r="B499" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="C499" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="500" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A500">
+        <v>88581</v>
+      </c>
+      <c r="B500" t="s">
+        <v>452</v>
+      </c>
+      <c r="C500" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="501" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A501">
+        <v>26492</v>
+      </c>
+      <c r="B501" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="C501" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="502" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B502" s="11" t="s">
+        <v>455</v>
+      </c>
+      <c r="C502" t="s">
+        <v>456</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>